<commit_message>
Update 생성형AI통합엔진 A2 IA v2 (xlsx)
</commit_message>
<xml_diff>
--- a/content/01_기획/2026-07-12_생성형AI통합엔진_A2_IA_v2.xlsx
+++ b/content/01_기획/2026-07-12_생성형AI통합엔진_A2_IA_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/seulking/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D51ED6-5202-474F-8178-910D8B24B07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F8C507-D974-4A48-9998-47C475D5D692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,14 +20,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">후속안건!$A$4:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">IA!$A$5:$L$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">IA!$A$5:$L$81</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="390">
   <si>
     <t>IA v2 개정안 요약</t>
   </si>
@@ -801,12 +801,6 @@
     <t>IA-040</t>
   </si>
   <si>
-    <t>queued</t>
-  </si>
-  <si>
-    <t>대기 중</t>
-  </si>
-  <si>
     <t>IA-041</t>
   </si>
   <si>
@@ -1142,9 +1136,6 @@
     <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
-    <t>IA-079</t>
-  </si>
-  <si>
     <t>이미지2 생성 화면 이동</t>
     <phoneticPr fontId="20" type="noConversion"/>
   </si>
@@ -1173,14 +1164,6 @@
     <phoneticPr fontId="20" type="noConversion"/>
   </si>
   <si>
-    <t>Kling auto, 16:9, 9:16, 4:3, 3:4, 1:1, 21:9 / Seedance auto, 16:9, 9:16, 1:1</t>
-    <phoneticPr fontId="20" type="noConversion"/>
-  </si>
-  <si>
-    <t>해상도 480p, 720p, 1080p, 4K (시연용)</t>
-    <phoneticPr fontId="20" type="noConversion"/>
-  </si>
-  <si>
     <t>현재 스탠다드 사용 중</t>
     <phoneticPr fontId="20" type="noConversion"/>
   </si>
@@ -1230,6 +1213,14 @@
   </si>
   <si>
     <t>찜 (좋아요)</t>
+    <phoneticPr fontId="20" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kling 16:9, 9:16, 1:1 / Seedance auto, 16:9, 9:16, 4:3, 3:4, 1:1, 21:9</t>
+    <phoneticPr fontId="20" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kling 1080p 고정 / Seedance 720p, 1080p</t>
     <phoneticPr fontId="20" type="noConversion"/>
   </si>
 </sst>
@@ -1886,7 +1877,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2118,6 +2109,12 @@
     </xf>
     <xf numFmtId="0" fontId="40" fillId="20" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2153,47 +2150,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2424,23 +2409,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
       <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="78" t="s">
+      <c r="A2" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
     </row>
     <row r="4" spans="1:6" ht="25.5" customHeight="1">
       <c r="A4" s="43" t="s">
@@ -2588,12 +2573,12 @@
       </c>
     </row>
     <row r="14" spans="1:6" ht="25.5" hidden="1" customHeight="1">
-      <c r="A14" s="81" t="s">
+      <c r="A14" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="82"/>
-      <c r="C14" s="82"/>
-      <c r="D14" s="83"/>
+      <c r="B14" s="84"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="85"/>
       <c r="E14" s="4">
         <v>78</v>
       </c>
@@ -2634,22 +2619,22 @@
     </row>
     <row r="2" spans="1:5" ht="17" customHeight="1"/>
     <row r="3" spans="1:5" ht="20" customHeight="1">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="86"/>
+      <c r="B3" s="87"/>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="88"/>
     </row>
     <row r="4" spans="1:5" ht="35" customHeight="1">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="86"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="88"/>
     </row>
     <row r="5" spans="1:5" s="32" customFormat="1" ht="17" customHeight="1">
       <c r="A5" s="22"/>
@@ -2781,29 +2766,29 @@
     <row r="14" spans="1:5" s="32" customFormat="1" ht="17" customHeight="1"/>
     <row r="15" spans="1:5" ht="17" customHeight="1"/>
     <row r="16" spans="1:5" ht="20" customHeight="1">
-      <c r="A16" s="84" t="s">
+      <c r="A16" s="86" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="85"/>
-      <c r="C16" s="85"/>
-      <c r="D16" s="85"/>
-      <c r="E16" s="86"/>
+      <c r="B16" s="87"/>
+      <c r="C16" s="87"/>
+      <c r="D16" s="87"/>
+      <c r="E16" s="88"/>
     </row>
     <row r="17" spans="1:5" ht="35" customHeight="1">
-      <c r="A17" s="88" t="s">
+      <c r="A17" s="90" t="s">
         <v>69</v>
       </c>
-      <c r="B17" s="85"/>
-      <c r="C17" s="85"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="86"/>
+      <c r="B17" s="87"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="87"/>
+      <c r="E17" s="88"/>
     </row>
     <row r="18" spans="1:5" ht="17" customHeight="1">
-      <c r="A18" s="89"/>
-      <c r="B18" s="90"/>
-      <c r="C18" s="90"/>
-      <c r="D18" s="90"/>
-      <c r="E18" s="91"/>
+      <c r="A18" s="91"/>
+      <c r="B18" s="92"/>
+      <c r="C18" s="92"/>
+      <c r="D18" s="92"/>
+      <c r="E18" s="93"/>
     </row>
     <row r="19" spans="1:5" ht="17" customHeight="1">
       <c r="A19" s="23" t="s">
@@ -2945,22 +2930,22 @@
     <row r="28" spans="1:5" s="32" customFormat="1" ht="17" customHeight="1"/>
     <row r="29" spans="1:5" ht="17" customHeight="1"/>
     <row r="30" spans="1:5" ht="20" customHeight="1">
-      <c r="A30" s="87" t="s">
+      <c r="A30" s="89" t="s">
         <v>99</v>
       </c>
-      <c r="B30" s="85"/>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="B30" s="87"/>
+      <c r="C30" s="87"/>
+      <c r="D30" s="87"/>
+      <c r="E30" s="88"/>
     </row>
     <row r="31" spans="1:5" s="33" customFormat="1" ht="35" customHeight="1">
-      <c r="A31" s="88" t="s">
+      <c r="A31" s="90" t="s">
         <v>100</v>
       </c>
-      <c r="B31" s="85"/>
-      <c r="C31" s="85"/>
-      <c r="D31" s="85"/>
-      <c r="E31" s="86"/>
+      <c r="B31" s="87"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="88"/>
     </row>
     <row r="32" spans="1:5" s="34" customFormat="1" ht="17" customHeight="1">
       <c r="A32" s="22"/>
@@ -3074,7 +3059,7 @@
   <sheetPr>
     <tabColor rgb="FF5B8DEF"/>
   </sheetPr>
-  <dimension ref="A1:N985"/>
+  <dimension ref="A1:N984"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6.6640625" style="14" bestFit="1" customWidth="1"/>
@@ -3113,38 +3098,38 @@
       <c r="M1" s="17"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="100" t="s">
+      <c r="A2" s="96" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
     </row>
     <row r="3" spans="1:14" ht="17" customHeight="1"/>
     <row r="4" spans="1:14" ht="19.5" customHeight="1">
       <c r="A4" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="101" t="s">
         <v>120</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="99" t="s">
+      <c r="C4" s="97"/>
+      <c r="D4" s="104" t="s">
         <v>121</v>
       </c>
-      <c r="E4" s="95"/>
-      <c r="F4" s="102" t="s">
+      <c r="E4" s="97"/>
+      <c r="F4" s="103" t="s">
         <v>122</v>
       </c>
-      <c r="G4" s="95"/>
+      <c r="G4" s="97"/>
     </row>
     <row r="5" spans="1:14" s="15" customFormat="1" ht="24" customHeight="1">
       <c r="A5" s="64" t="s">
@@ -3191,10 +3176,10 @@
       <c r="A6" s="72" t="s">
         <v>133</v>
       </c>
-      <c r="B6" s="92" t="s">
+      <c r="B6" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="92" t="s">
+      <c r="C6" s="94" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="73" t="s">
@@ -3218,8 +3203,8 @@
       <c r="A7" s="72" t="s">
         <v>136</v>
       </c>
-      <c r="B7" s="93"/>
-      <c r="C7" s="93"/>
+      <c r="B7" s="95"/>
+      <c r="C7" s="95"/>
       <c r="D7" s="73" t="s">
         <v>137</v>
       </c>
@@ -3239,13 +3224,13 @@
       <c r="A8" s="72" t="s">
         <v>138</v>
       </c>
-      <c r="B8" s="92" t="s">
+      <c r="B8" s="94" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="94" t="s">
         <v>139</v>
       </c>
-      <c r="D8" s="92" t="s">
+      <c r="D8" s="94" t="s">
         <v>10</v>
       </c>
       <c r="E8" s="74"/>
@@ -3266,10 +3251,10 @@
       <c r="A9" s="72" t="s">
         <v>141</v>
       </c>
-      <c r="B9" s="93"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="93"/>
-      <c r="E9" s="96" t="s">
+      <c r="B9" s="95"/>
+      <c r="C9" s="95"/>
+      <c r="D9" s="95"/>
+      <c r="E9" s="99" t="s">
         <v>142</v>
       </c>
       <c r="F9" s="73" t="s">
@@ -3293,10 +3278,10 @@
       <c r="A10" s="72" t="s">
         <v>145</v>
       </c>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="97"/>
+      <c r="B10" s="95"/>
+      <c r="C10" s="95"/>
+      <c r="D10" s="95"/>
+      <c r="E10" s="102"/>
       <c r="F10" s="73" t="s">
         <v>146</v>
       </c>
@@ -3311,19 +3296,19 @@
         <v>147</v>
       </c>
       <c r="M10" s="69" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="11" spans="1:14" s="67" customFormat="1" ht="21" customHeight="1">
       <c r="A11" s="72" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="93"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="93"/>
-      <c r="E11" s="97"/>
+      <c r="B11" s="95"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="95"/>
+      <c r="E11" s="102"/>
       <c r="F11" s="73" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="G11" s="74"/>
       <c r="H11" s="74"/>
@@ -3333,20 +3318,20 @@
       </c>
       <c r="K11" s="69"/>
       <c r="L11" s="68" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="M11" s="69" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="21" customHeight="1">
       <c r="A12" s="72" t="s">
         <v>151</v>
       </c>
-      <c r="B12" s="93"/>
-      <c r="C12" s="93"/>
-      <c r="D12" s="93"/>
-      <c r="E12" s="97"/>
+      <c r="B12" s="95"/>
+      <c r="C12" s="95"/>
+      <c r="D12" s="95"/>
+      <c r="E12" s="102"/>
       <c r="F12" s="73" t="s">
         <v>149</v>
       </c>
@@ -3366,15 +3351,15 @@
       <c r="A13" s="72" t="s">
         <v>154</v>
       </c>
-      <c r="B13" s="93"/>
-      <c r="C13" s="93"/>
-      <c r="D13" s="93"/>
-      <c r="E13" s="97"/>
+      <c r="B13" s="95"/>
+      <c r="C13" s="95"/>
+      <c r="D13" s="95"/>
+      <c r="E13" s="102"/>
       <c r="F13" s="73" t="s">
         <v>152</v>
       </c>
       <c r="G13" s="73" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="H13" s="74"/>
       <c r="I13" s="68"/>
@@ -3388,16 +3373,16 @@
       <c r="M13" s="69"/>
       <c r="N13" s="13"/>
     </row>
-    <row r="14" spans="1:14" s="104" customFormat="1" ht="21" customHeight="1">
+    <row r="14" spans="1:14" s="67" customFormat="1" ht="21" customHeight="1">
       <c r="A14" s="72" t="s">
         <v>158</v>
       </c>
-      <c r="B14" s="93"/>
-      <c r="C14" s="93"/>
-      <c r="D14" s="93"/>
-      <c r="E14" s="98"/>
+      <c r="B14" s="95"/>
+      <c r="C14" s="95"/>
+      <c r="D14" s="95"/>
+      <c r="E14" s="100"/>
       <c r="F14" s="73" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="G14" s="74"/>
       <c r="H14" s="74"/>
@@ -3406,20 +3391,20 @@
         <v>8</v>
       </c>
       <c r="K14" s="69" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="L14" s="68"/>
       <c r="M14" s="69"/>
-      <c r="N14" s="106"/>
+      <c r="N14" s="79"/>
     </row>
     <row r="15" spans="1:14" ht="21" customHeight="1">
       <c r="A15" s="72" t="s">
         <v>160</v>
       </c>
-      <c r="B15" s="93"/>
-      <c r="C15" s="93"/>
-      <c r="D15" s="93"/>
-      <c r="E15" s="96" t="s">
+      <c r="B15" s="95"/>
+      <c r="C15" s="95"/>
+      <c r="D15" s="95"/>
+      <c r="E15" s="99" t="s">
         <v>155</v>
       </c>
       <c r="F15" s="73" t="s">
@@ -3441,12 +3426,12 @@
       <c r="A16" s="72" t="s">
         <v>162</v>
       </c>
-      <c r="B16" s="93"/>
-      <c r="C16" s="93"/>
-      <c r="D16" s="93"/>
-      <c r="E16" s="97"/>
+      <c r="B16" s="95"/>
+      <c r="C16" s="95"/>
+      <c r="D16" s="95"/>
+      <c r="E16" s="102"/>
       <c r="F16" s="73" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="G16" s="74"/>
       <c r="H16" s="74"/>
@@ -3466,12 +3451,12 @@
       <c r="A17" s="72" t="s">
         <v>166</v>
       </c>
-      <c r="B17" s="93"/>
-      <c r="C17" s="93"/>
-      <c r="D17" s="93"/>
-      <c r="E17" s="97"/>
+      <c r="B17" s="95"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="95"/>
+      <c r="E17" s="102"/>
       <c r="F17" s="73" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="G17" s="74"/>
       <c r="H17" s="74"/>
@@ -3481,7 +3466,7 @@
       </c>
       <c r="K17" s="69"/>
       <c r="L17" s="68" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="M17" s="69"/>
     </row>
@@ -3489,10 +3474,10 @@
       <c r="A18" s="72" t="s">
         <v>169</v>
       </c>
-      <c r="B18" s="93"/>
-      <c r="C18" s="93"/>
-      <c r="D18" s="93"/>
-      <c r="E18" s="97"/>
+      <c r="B18" s="95"/>
+      <c r="C18" s="95"/>
+      <c r="D18" s="95"/>
+      <c r="E18" s="102"/>
       <c r="F18" s="73" t="s">
         <v>161</v>
       </c>
@@ -3512,10 +3497,10 @@
       <c r="A19" s="72" t="s">
         <v>171</v>
       </c>
-      <c r="B19" s="93"/>
-      <c r="C19" s="93"/>
-      <c r="D19" s="93"/>
-      <c r="E19" s="97"/>
+      <c r="B19" s="95"/>
+      <c r="C19" s="95"/>
+      <c r="D19" s="95"/>
+      <c r="E19" s="102"/>
       <c r="F19" s="73" t="s">
         <v>163</v>
       </c>
@@ -3537,10 +3522,10 @@
       <c r="A20" s="72" t="s">
         <v>175</v>
       </c>
-      <c r="B20" s="93"/>
-      <c r="C20" s="93"/>
-      <c r="D20" s="93"/>
-      <c r="E20" s="98"/>
+      <c r="B20" s="95"/>
+      <c r="C20" s="95"/>
+      <c r="D20" s="95"/>
+      <c r="E20" s="100"/>
       <c r="F20" s="71" t="s">
         <v>167</v>
       </c>
@@ -3562,13 +3547,13 @@
       <c r="A21" s="72" t="s">
         <v>179</v>
       </c>
-      <c r="B21" s="92" t="s">
+      <c r="B21" s="94" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="92" t="s">
+      <c r="C21" s="94" t="s">
         <v>139</v>
       </c>
-      <c r="D21" s="92" t="s">
+      <c r="D21" s="94" t="s">
         <v>12</v>
       </c>
       <c r="E21" s="75"/>
@@ -3591,10 +3576,10 @@
       <c r="A22" s="72" t="s">
         <v>182</v>
       </c>
-      <c r="B22" s="93"/>
-      <c r="C22" s="93"/>
-      <c r="D22" s="93"/>
-      <c r="E22" s="92" t="s">
+      <c r="B22" s="95"/>
+      <c r="C22" s="95"/>
+      <c r="D22" s="95"/>
+      <c r="E22" s="94" t="s">
         <v>172</v>
       </c>
       <c r="F22" s="73" t="s">
@@ -3618,11 +3603,11 @@
       <c r="A23" s="72" t="s">
         <v>187</v>
       </c>
-      <c r="B23" s="93"/>
-      <c r="C23" s="93"/>
-      <c r="D23" s="93"/>
-      <c r="E23" s="93"/>
-      <c r="F23" s="92" t="s">
+      <c r="B23" s="95"/>
+      <c r="C23" s="95"/>
+      <c r="D23" s="95"/>
+      <c r="E23" s="95"/>
+      <c r="F23" s="94" t="s">
         <v>176</v>
       </c>
       <c r="G23" s="73" t="s">
@@ -3643,11 +3628,11 @@
       <c r="A24" s="72" t="s">
         <v>191</v>
       </c>
-      <c r="B24" s="93"/>
-      <c r="C24" s="93"/>
-      <c r="D24" s="93"/>
-      <c r="E24" s="93"/>
-      <c r="F24" s="93"/>
+      <c r="B24" s="95"/>
+      <c r="C24" s="95"/>
+      <c r="D24" s="95"/>
+      <c r="E24" s="95"/>
+      <c r="F24" s="95"/>
       <c r="G24" s="73" t="s">
         <v>180</v>
       </c>
@@ -3666,11 +3651,11 @@
       <c r="A25" s="72" t="s">
         <v>193</v>
       </c>
-      <c r="B25" s="93"/>
-      <c r="C25" s="93"/>
-      <c r="D25" s="93"/>
-      <c r="E25" s="93"/>
-      <c r="F25" s="92" t="s">
+      <c r="B25" s="95"/>
+      <c r="C25" s="95"/>
+      <c r="D25" s="95"/>
+      <c r="E25" s="95"/>
+      <c r="F25" s="94" t="s">
         <v>183</v>
       </c>
       <c r="G25" s="73" t="s">
@@ -3693,11 +3678,11 @@
       <c r="A26" s="72" t="s">
         <v>196</v>
       </c>
-      <c r="B26" s="93"/>
-      <c r="C26" s="93"/>
-      <c r="D26" s="93"/>
-      <c r="E26" s="93"/>
-      <c r="F26" s="93"/>
+      <c r="B26" s="95"/>
+      <c r="C26" s="95"/>
+      <c r="D26" s="95"/>
+      <c r="E26" s="95"/>
+      <c r="F26" s="95"/>
       <c r="G26" s="71" t="s">
         <v>188</v>
       </c>
@@ -3718,10 +3703,10 @@
       <c r="A27" s="72" t="s">
         <v>199</v>
       </c>
-      <c r="B27" s="93"/>
-      <c r="C27" s="93"/>
-      <c r="D27" s="93"/>
-      <c r="E27" s="93"/>
+      <c r="B27" s="95"/>
+      <c r="C27" s="95"/>
+      <c r="D27" s="95"/>
+      <c r="E27" s="95"/>
       <c r="F27" s="73" t="s">
         <v>192</v>
       </c>
@@ -3732,7 +3717,7 @@
         <v>8</v>
       </c>
       <c r="K27" s="69" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="L27" s="68"/>
       <c r="M27" s="69"/>
@@ -3741,11 +3726,11 @@
       <c r="A28" s="72" t="s">
         <v>205</v>
       </c>
-      <c r="B28" s="93"/>
-      <c r="C28" s="93"/>
-      <c r="D28" s="93"/>
-      <c r="E28" s="93"/>
-      <c r="F28" s="92" t="s">
+      <c r="B28" s="95"/>
+      <c r="C28" s="95"/>
+      <c r="D28" s="95"/>
+      <c r="E28" s="95"/>
+      <c r="F28" s="94" t="s">
         <v>194</v>
       </c>
       <c r="G28" s="73" t="s">
@@ -3764,11 +3749,11 @@
       <c r="A29" s="72" t="s">
         <v>208</v>
       </c>
-      <c r="B29" s="93"/>
-      <c r="C29" s="93"/>
-      <c r="D29" s="93"/>
-      <c r="E29" s="93"/>
-      <c r="F29" s="93"/>
+      <c r="B29" s="95"/>
+      <c r="C29" s="95"/>
+      <c r="D29" s="95"/>
+      <c r="E29" s="95"/>
+      <c r="F29" s="95"/>
       <c r="G29" s="73" t="s">
         <v>197</v>
       </c>
@@ -3787,13 +3772,13 @@
       <c r="A30" s="72" t="s">
         <v>210</v>
       </c>
-      <c r="B30" s="93"/>
-      <c r="C30" s="93"/>
-      <c r="D30" s="93"/>
-      <c r="E30" s="92" t="s">
+      <c r="B30" s="95"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="95"/>
+      <c r="E30" s="94" t="s">
         <v>200</v>
       </c>
-      <c r="F30" s="92" t="s">
+      <c r="F30" s="94" t="s">
         <v>201</v>
       </c>
       <c r="G30" s="73" t="s">
@@ -3818,11 +3803,11 @@
       <c r="A31" s="72" t="s">
         <v>212</v>
       </c>
-      <c r="B31" s="93"/>
-      <c r="C31" s="93"/>
-      <c r="D31" s="93"/>
-      <c r="E31" s="93"/>
-      <c r="F31" s="93"/>
+      <c r="B31" s="95"/>
+      <c r="C31" s="95"/>
+      <c r="D31" s="95"/>
+      <c r="E31" s="95"/>
+      <c r="F31" s="95"/>
       <c r="G31" s="71" t="s">
         <v>206</v>
       </c>
@@ -3834,7 +3819,7 @@
         <v>8</v>
       </c>
       <c r="K31" s="69" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="L31" s="68"/>
       <c r="M31" s="69"/>
@@ -3843,10 +3828,10 @@
       <c r="A32" s="72" t="s">
         <v>215</v>
       </c>
-      <c r="B32" s="93"/>
-      <c r="C32" s="93"/>
-      <c r="D32" s="93"/>
-      <c r="E32" s="93"/>
+      <c r="B32" s="95"/>
+      <c r="C32" s="95"/>
+      <c r="D32" s="95"/>
+      <c r="E32" s="95"/>
       <c r="F32" s="73" t="s">
         <v>176</v>
       </c>
@@ -3866,10 +3851,10 @@
       <c r="A33" s="72" t="s">
         <v>220</v>
       </c>
-      <c r="B33" s="93"/>
-      <c r="C33" s="93"/>
-      <c r="D33" s="93"/>
-      <c r="E33" s="93"/>
+      <c r="B33" s="95"/>
+      <c r="C33" s="95"/>
+      <c r="D33" s="95"/>
+      <c r="E33" s="95"/>
       <c r="F33" s="73" t="s">
         <v>192</v>
       </c>
@@ -3890,10 +3875,10 @@
       <c r="A34" s="72" t="s">
         <v>223</v>
       </c>
-      <c r="B34" s="93"/>
-      <c r="C34" s="93"/>
-      <c r="D34" s="93"/>
-      <c r="E34" s="93"/>
+      <c r="B34" s="95"/>
+      <c r="C34" s="95"/>
+      <c r="D34" s="95"/>
+      <c r="E34" s="95"/>
       <c r="F34" s="73" t="s">
         <v>194</v>
       </c>
@@ -3916,10 +3901,10 @@
       <c r="A35" s="72" t="s">
         <v>226</v>
       </c>
-      <c r="B35" s="93"/>
-      <c r="C35" s="93"/>
-      <c r="D35" s="93"/>
-      <c r="E35" s="96" t="s">
+      <c r="B35" s="95"/>
+      <c r="C35" s="95"/>
+      <c r="D35" s="95"/>
+      <c r="E35" s="99" t="s">
         <v>216</v>
       </c>
       <c r="F35" s="73" t="s">
@@ -3945,10 +3930,10 @@
       <c r="A36" s="72" t="s">
         <v>229</v>
       </c>
-      <c r="B36" s="93"/>
-      <c r="C36" s="93"/>
-      <c r="D36" s="93"/>
-      <c r="E36" s="97"/>
+      <c r="B36" s="95"/>
+      <c r="C36" s="95"/>
+      <c r="D36" s="95"/>
+      <c r="E36" s="102"/>
       <c r="F36" s="73" t="s">
         <v>221</v>
       </c>
@@ -3968,10 +3953,10 @@
       <c r="A37" s="72" t="s">
         <v>232</v>
       </c>
-      <c r="B37" s="93"/>
-      <c r="C37" s="93"/>
-      <c r="D37" s="93"/>
-      <c r="E37" s="97"/>
+      <c r="B37" s="95"/>
+      <c r="C37" s="95"/>
+      <c r="D37" s="95"/>
+      <c r="E37" s="102"/>
       <c r="F37" s="73" t="s">
         <v>224</v>
       </c>
@@ -3991,10 +3976,10 @@
       <c r="A38" s="72" t="s">
         <v>235</v>
       </c>
-      <c r="B38" s="93"/>
-      <c r="C38" s="93"/>
-      <c r="D38" s="93"/>
-      <c r="E38" s="97"/>
+      <c r="B38" s="95"/>
+      <c r="C38" s="95"/>
+      <c r="D38" s="95"/>
+      <c r="E38" s="102"/>
       <c r="F38" s="73" t="s">
         <v>227</v>
       </c>
@@ -4014,10 +3999,10 @@
       <c r="A39" s="72" t="s">
         <v>237</v>
       </c>
-      <c r="B39" s="93"/>
-      <c r="C39" s="93"/>
-      <c r="D39" s="93"/>
-      <c r="E39" s="97"/>
+      <c r="B39" s="95"/>
+      <c r="C39" s="95"/>
+      <c r="D39" s="95"/>
+      <c r="E39" s="102"/>
       <c r="F39" s="73" t="s">
         <v>230</v>
       </c>
@@ -4037,10 +4022,10 @@
       <c r="A40" s="72" t="s">
         <v>241</v>
       </c>
-      <c r="B40" s="93"/>
-      <c r="C40" s="93"/>
-      <c r="D40" s="93"/>
-      <c r="E40" s="98"/>
+      <c r="B40" s="95"/>
+      <c r="C40" s="95"/>
+      <c r="D40" s="95"/>
+      <c r="E40" s="100"/>
       <c r="F40" s="71" t="s">
         <v>233</v>
       </c>
@@ -4060,13 +4045,13 @@
       <c r="A41" s="72" t="s">
         <v>243</v>
       </c>
-      <c r="B41" s="92" t="s">
+      <c r="B41" s="94" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="92" t="s">
+      <c r="C41" s="94" t="s">
         <v>139</v>
       </c>
-      <c r="D41" s="92" t="s">
+      <c r="D41" s="94" t="s">
         <v>15</v>
       </c>
       <c r="E41" s="75"/>
@@ -4089,9 +4074,9 @@
       <c r="A42" s="72" t="s">
         <v>246</v>
       </c>
-      <c r="B42" s="93"/>
-      <c r="C42" s="93"/>
-      <c r="D42" s="93"/>
+      <c r="B42" s="95"/>
+      <c r="C42" s="95"/>
+      <c r="D42" s="95"/>
       <c r="E42" s="73" t="s">
         <v>238</v>
       </c>
@@ -4114,9 +4099,9 @@
       <c r="A43" s="72" t="s">
         <v>249</v>
       </c>
-      <c r="B43" s="93"/>
-      <c r="C43" s="93"/>
-      <c r="D43" s="93"/>
+      <c r="B43" s="95"/>
+      <c r="C43" s="95"/>
+      <c r="D43" s="95"/>
       <c r="E43" s="73" t="s">
         <v>242</v>
       </c>
@@ -4135,17 +4120,17 @@
       <c r="A44" s="72" t="s">
         <v>253</v>
       </c>
-      <c r="B44" s="93"/>
-      <c r="C44" s="93"/>
-      <c r="D44" s="93"/>
-      <c r="E44" s="96" t="s">
+      <c r="B44" s="95"/>
+      <c r="C44" s="95"/>
+      <c r="D44" s="95"/>
+      <c r="E44" s="99" t="s">
         <v>183</v>
       </c>
-      <c r="F44" s="96" t="s">
+      <c r="F44" s="99" t="s">
         <v>244</v>
       </c>
       <c r="G44" s="73" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="H44" s="75"/>
       <c r="I44" s="68"/>
@@ -4157,18 +4142,18 @@
       </c>
       <c r="L44" s="68"/>
       <c r="M44" s="69" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="21" customHeight="1">
       <c r="A45" s="72" t="s">
         <v>256</v>
       </c>
-      <c r="B45" s="93"/>
-      <c r="C45" s="93"/>
-      <c r="D45" s="93"/>
-      <c r="E45" s="97"/>
-      <c r="F45" s="98"/>
+      <c r="B45" s="95"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="102"/>
+      <c r="F45" s="100"/>
       <c r="G45" s="73" t="s">
         <v>247</v>
       </c>
@@ -4185,12 +4170,12 @@
     </row>
     <row r="46" spans="1:14" ht="21" customHeight="1">
       <c r="A46" s="72" t="s">
-        <v>259</v>
-      </c>
-      <c r="B46" s="93"/>
-      <c r="C46" s="93"/>
-      <c r="D46" s="93"/>
-      <c r="E46" s="97"/>
+        <v>257</v>
+      </c>
+      <c r="B46" s="95"/>
+      <c r="C46" s="95"/>
+      <c r="D46" s="95"/>
+      <c r="E46" s="102"/>
       <c r="F46" s="71" t="s">
         <v>250</v>
       </c>
@@ -4208,19 +4193,19 @@
       <c r="L46" s="68"/>
       <c r="M46" s="69"/>
     </row>
-    <row r="47" spans="1:14" s="104" customFormat="1" ht="21" customHeight="1">
+    <row r="47" spans="1:14" s="67" customFormat="1" ht="21" customHeight="1">
       <c r="A47" s="72" t="s">
-        <v>262</v>
-      </c>
-      <c r="B47" s="93"/>
-      <c r="C47" s="93"/>
-      <c r="D47" s="93"/>
-      <c r="E47" s="97"/>
+        <v>260</v>
+      </c>
+      <c r="B47" s="95"/>
+      <c r="C47" s="95"/>
+      <c r="D47" s="95"/>
+      <c r="E47" s="102"/>
       <c r="F47" s="71" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="G47" s="71" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
       <c r="H47" s="75"/>
       <c r="I47" s="68"/>
@@ -4233,19 +4218,19 @@
       <c r="L47" s="68"/>
       <c r="M47" s="69"/>
     </row>
-    <row r="48" spans="1:14" s="104" customFormat="1" ht="21" customHeight="1">
+    <row r="48" spans="1:14" s="67" customFormat="1" ht="21" customHeight="1">
       <c r="A48" s="72" t="s">
-        <v>265</v>
-      </c>
-      <c r="B48" s="93"/>
-      <c r="C48" s="93"/>
-      <c r="D48" s="93"/>
-      <c r="E48" s="98"/>
+        <v>263</v>
+      </c>
+      <c r="B48" s="95"/>
+      <c r="C48" s="95"/>
+      <c r="D48" s="95"/>
+      <c r="E48" s="100"/>
       <c r="F48" s="71" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="G48" s="71" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
       <c r="H48" s="75"/>
       <c r="I48" s="68"/>
@@ -4260,11 +4245,11 @@
     </row>
     <row r="49" spans="1:13" ht="21" customHeight="1">
       <c r="A49" s="72" t="s">
-        <v>268</v>
-      </c>
-      <c r="B49" s="93"/>
-      <c r="C49" s="93"/>
-      <c r="D49" s="93"/>
+        <v>266</v>
+      </c>
+      <c r="B49" s="95"/>
+      <c r="C49" s="95"/>
+      <c r="D49" s="95"/>
       <c r="E49" s="73" t="s">
         <v>254</v>
       </c>
@@ -4283,19 +4268,19 @@
     </row>
     <row r="50" spans="1:13" ht="21" customHeight="1">
       <c r="A50" s="72" t="s">
-        <v>271</v>
-      </c>
-      <c r="B50" s="93"/>
-      <c r="C50" s="93"/>
-      <c r="D50" s="93"/>
-      <c r="E50" s="92" t="s">
+        <v>269</v>
+      </c>
+      <c r="B50" s="95"/>
+      <c r="C50" s="95"/>
+      <c r="D50" s="95"/>
+      <c r="E50" s="99" t="s">
         <v>192</v>
       </c>
       <c r="F50" s="73" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G50" s="73" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="H50" s="75"/>
       <c r="I50" s="68"/>
@@ -4308,17 +4293,17 @@
     </row>
     <row r="51" spans="1:13" ht="21" customHeight="1">
       <c r="A51" s="72" t="s">
-        <v>274</v>
-      </c>
-      <c r="B51" s="93"/>
-      <c r="C51" s="93"/>
-      <c r="D51" s="93"/>
-      <c r="E51" s="93"/>
+        <v>272</v>
+      </c>
+      <c r="B51" s="95"/>
+      <c r="C51" s="95"/>
+      <c r="D51" s="95"/>
+      <c r="E51" s="102"/>
       <c r="F51" s="73" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G51" s="73" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H51" s="75"/>
       <c r="I51" s="68"/>
@@ -4331,17 +4316,17 @@
     </row>
     <row r="52" spans="1:13" ht="21" customHeight="1">
       <c r="A52" s="72" t="s">
-        <v>275</v>
-      </c>
-      <c r="B52" s="93"/>
-      <c r="C52" s="93"/>
-      <c r="D52" s="93"/>
-      <c r="E52" s="93"/>
-      <c r="F52" s="73" t="s">
-        <v>263</v>
-      </c>
-      <c r="G52" s="73" t="s">
+        <v>273</v>
+      </c>
+      <c r="B52" s="95"/>
+      <c r="C52" s="95"/>
+      <c r="D52" s="95"/>
+      <c r="E52" s="100"/>
+      <c r="F52" s="71" t="s">
         <v>264</v>
+      </c>
+      <c r="G52" s="71" t="s">
+        <v>265</v>
       </c>
       <c r="H52" s="75"/>
       <c r="I52" s="68"/>
@@ -4354,38 +4339,40 @@
     </row>
     <row r="53" spans="1:13" ht="21" customHeight="1">
       <c r="A53" s="72" t="s">
-        <v>276</v>
-      </c>
-      <c r="B53" s="93"/>
-      <c r="C53" s="93"/>
-      <c r="D53" s="93"/>
-      <c r="E53" s="93"/>
-      <c r="F53" s="71" t="s">
-        <v>266</v>
-      </c>
-      <c r="G53" s="71" t="s">
+        <v>274</v>
+      </c>
+      <c r="B53" s="95"/>
+      <c r="C53" s="95"/>
+      <c r="D53" s="95"/>
+      <c r="E53" s="73" t="s">
         <v>267</v>
       </c>
+      <c r="F53" s="75"/>
+      <c r="G53" s="75"/>
       <c r="H53" s="75"/>
       <c r="I53" s="68"/>
       <c r="J53" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="K53" s="69"/>
+      <c r="K53" s="69" t="s">
+        <v>268</v>
+      </c>
       <c r="L53" s="68"/>
       <c r="M53" s="69"/>
     </row>
     <row r="54" spans="1:13" ht="21" customHeight="1">
       <c r="A54" s="72" t="s">
-        <v>277</v>
-      </c>
-      <c r="B54" s="93"/>
-      <c r="C54" s="93"/>
-      <c r="D54" s="93"/>
-      <c r="E54" s="73" t="s">
-        <v>269</v>
-      </c>
-      <c r="F54" s="75"/>
+        <v>275</v>
+      </c>
+      <c r="B54" s="95"/>
+      <c r="C54" s="95"/>
+      <c r="D54" s="95"/>
+      <c r="E54" s="99" t="s">
+        <v>270</v>
+      </c>
+      <c r="F54" s="73" t="s">
+        <v>217</v>
+      </c>
       <c r="G54" s="75"/>
       <c r="H54" s="75"/>
       <c r="I54" s="68"/>
@@ -4393,23 +4380,23 @@
         <v>8</v>
       </c>
       <c r="K54" s="69" t="s">
-        <v>270</v>
-      </c>
-      <c r="L54" s="68"/>
+        <v>271</v>
+      </c>
+      <c r="L54" s="68" t="s">
+        <v>219</v>
+      </c>
       <c r="M54" s="69"/>
     </row>
     <row r="55" spans="1:13" ht="21" customHeight="1">
       <c r="A55" s="72" t="s">
-        <v>278</v>
-      </c>
-      <c r="B55" s="93"/>
-      <c r="C55" s="93"/>
-      <c r="D55" s="93"/>
-      <c r="E55" s="96" t="s">
-        <v>272</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="B55" s="95"/>
+      <c r="C55" s="95"/>
+      <c r="D55" s="95"/>
+      <c r="E55" s="102"/>
       <c r="F55" s="73" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="G55" s="75"/>
       <c r="H55" s="75"/>
@@ -4418,23 +4405,21 @@
         <v>8</v>
       </c>
       <c r="K55" s="69" t="s">
-        <v>273</v>
-      </c>
-      <c r="L55" s="68" t="s">
-        <v>219</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="L55" s="68"/>
       <c r="M55" s="69"/>
     </row>
     <row r="56" spans="1:13" ht="21" customHeight="1">
       <c r="A56" s="72" t="s">
-        <v>279</v>
-      </c>
-      <c r="B56" s="93"/>
-      <c r="C56" s="93"/>
-      <c r="D56" s="93"/>
-      <c r="E56" s="97"/>
+        <v>277</v>
+      </c>
+      <c r="B56" s="95"/>
+      <c r="C56" s="95"/>
+      <c r="D56" s="95"/>
+      <c r="E56" s="102"/>
       <c r="F56" s="73" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="G56" s="75"/>
       <c r="H56" s="75"/>
@@ -4443,21 +4428,21 @@
         <v>8</v>
       </c>
       <c r="K56" s="69" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="L56" s="68"/>
       <c r="M56" s="69"/>
     </row>
     <row r="57" spans="1:13" ht="21" customHeight="1">
       <c r="A57" s="72" t="s">
-        <v>281</v>
-      </c>
-      <c r="B57" s="93"/>
-      <c r="C57" s="93"/>
-      <c r="D57" s="93"/>
-      <c r="E57" s="97"/>
+        <v>279</v>
+      </c>
+      <c r="B57" s="95"/>
+      <c r="C57" s="95"/>
+      <c r="D57" s="95"/>
+      <c r="E57" s="102"/>
       <c r="F57" s="73" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="G57" s="75"/>
       <c r="H57" s="75"/>
@@ -4466,21 +4451,21 @@
         <v>8</v>
       </c>
       <c r="K57" s="69" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="L57" s="68"/>
       <c r="M57" s="69"/>
     </row>
     <row r="58" spans="1:13" ht="21" customHeight="1">
       <c r="A58" s="72" t="s">
-        <v>284</v>
-      </c>
-      <c r="B58" s="93"/>
-      <c r="C58" s="93"/>
-      <c r="D58" s="93"/>
-      <c r="E58" s="97"/>
+        <v>282</v>
+      </c>
+      <c r="B58" s="95"/>
+      <c r="C58" s="95"/>
+      <c r="D58" s="95"/>
+      <c r="E58" s="102"/>
       <c r="F58" s="73" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G58" s="75"/>
       <c r="H58" s="75"/>
@@ -4489,21 +4474,21 @@
         <v>8</v>
       </c>
       <c r="K58" s="69" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="L58" s="68"/>
       <c r="M58" s="69"/>
     </row>
     <row r="59" spans="1:13" ht="21" customHeight="1">
       <c r="A59" s="72" t="s">
-        <v>288</v>
-      </c>
-      <c r="B59" s="93"/>
-      <c r="C59" s="93"/>
-      <c r="D59" s="93"/>
-      <c r="E59" s="97"/>
-      <c r="F59" s="73" t="s">
-        <v>230</v>
+        <v>286</v>
+      </c>
+      <c r="B59" s="95"/>
+      <c r="C59" s="95"/>
+      <c r="D59" s="95"/>
+      <c r="E59" s="100"/>
+      <c r="F59" s="71" t="s">
+        <v>233</v>
       </c>
       <c r="G59" s="75"/>
       <c r="H59" s="75"/>
@@ -4512,74 +4497,76 @@
         <v>8</v>
       </c>
       <c r="K59" s="69" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="L59" s="68"/>
       <c r="M59" s="69"/>
     </row>
     <row r="60" spans="1:13" ht="21" customHeight="1">
       <c r="A60" s="72" t="s">
-        <v>289</v>
-      </c>
-      <c r="B60" s="93"/>
-      <c r="C60" s="93"/>
-      <c r="D60" s="93"/>
-      <c r="E60" s="98"/>
-      <c r="F60" s="71" t="s">
-        <v>233</v>
-      </c>
+        <v>287</v>
+      </c>
+      <c r="B60" s="94" t="s">
+        <v>18</v>
+      </c>
+      <c r="C60" s="94" t="s">
+        <v>139</v>
+      </c>
+      <c r="D60" s="94" t="s">
+        <v>18</v>
+      </c>
+      <c r="E60" s="75"/>
+      <c r="F60" s="75"/>
       <c r="G60" s="75"/>
       <c r="H60" s="75"/>
-      <c r="I60" s="68"/>
+      <c r="I60" s="68" t="s">
+        <v>19</v>
+      </c>
       <c r="J60" s="76" t="s">
         <v>8</v>
       </c>
       <c r="K60" s="69" t="s">
-        <v>234</v>
+        <v>278</v>
       </c>
       <c r="L60" s="68"/>
       <c r="M60" s="69"/>
     </row>
     <row r="61" spans="1:13" ht="21" customHeight="1">
       <c r="A61" s="72" t="s">
-        <v>290</v>
-      </c>
-      <c r="B61" s="92" t="s">
-        <v>18</v>
-      </c>
-      <c r="C61" s="92" t="s">
-        <v>139</v>
-      </c>
-      <c r="D61" s="92" t="s">
-        <v>18</v>
-      </c>
-      <c r="E61" s="75"/>
+        <v>288</v>
+      </c>
+      <c r="B61" s="95"/>
+      <c r="C61" s="95"/>
+      <c r="D61" s="95"/>
+      <c r="E61" s="73" t="s">
+        <v>280</v>
+      </c>
       <c r="F61" s="75"/>
       <c r="G61" s="75"/>
       <c r="H61" s="75"/>
-      <c r="I61" s="68" t="s">
-        <v>19</v>
-      </c>
+      <c r="I61" s="68"/>
       <c r="J61" s="76" t="s">
         <v>8</v>
       </c>
       <c r="K61" s="69" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="L61" s="68"/>
       <c r="M61" s="69"/>
     </row>
     <row r="62" spans="1:13" ht="21" customHeight="1">
       <c r="A62" s="72" t="s">
-        <v>293</v>
-      </c>
-      <c r="B62" s="93"/>
-      <c r="C62" s="93"/>
-      <c r="D62" s="93"/>
-      <c r="E62" s="73" t="s">
-        <v>282</v>
-      </c>
-      <c r="F62" s="75"/>
+        <v>291</v>
+      </c>
+      <c r="B62" s="95"/>
+      <c r="C62" s="95"/>
+      <c r="D62" s="95"/>
+      <c r="E62" s="94" t="s">
+        <v>283</v>
+      </c>
+      <c r="F62" s="73" t="s">
+        <v>284</v>
+      </c>
       <c r="G62" s="75"/>
       <c r="H62" s="75"/>
       <c r="I62" s="68"/>
@@ -4587,23 +4574,21 @@
         <v>8</v>
       </c>
       <c r="K62" s="69" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L62" s="68"/>
       <c r="M62" s="69"/>
     </row>
     <row r="63" spans="1:13" ht="21" customHeight="1">
       <c r="A63" s="72" t="s">
-        <v>297</v>
-      </c>
-      <c r="B63" s="93"/>
-      <c r="C63" s="93"/>
-      <c r="D63" s="93"/>
-      <c r="E63" s="92" t="s">
-        <v>285</v>
-      </c>
+        <v>295</v>
+      </c>
+      <c r="B63" s="95"/>
+      <c r="C63" s="95"/>
+      <c r="D63" s="95"/>
+      <c r="E63" s="95"/>
       <c r="F63" s="73" t="s">
-        <v>286</v>
+        <v>146</v>
       </c>
       <c r="G63" s="75"/>
       <c r="H63" s="75"/>
@@ -4611,22 +4596,20 @@
       <c r="J63" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="K63" s="69" t="s">
-        <v>287</v>
-      </c>
+      <c r="K63" s="69"/>
       <c r="L63" s="68"/>
       <c r="M63" s="69"/>
     </row>
     <row r="64" spans="1:13" ht="21" customHeight="1">
       <c r="A64" s="72" t="s">
-        <v>301</v>
-      </c>
-      <c r="B64" s="93"/>
-      <c r="C64" s="93"/>
-      <c r="D64" s="93"/>
-      <c r="E64" s="93"/>
+        <v>299</v>
+      </c>
+      <c r="B64" s="95"/>
+      <c r="C64" s="95"/>
+      <c r="D64" s="95"/>
+      <c r="E64" s="95"/>
       <c r="F64" s="73" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="G64" s="75"/>
       <c r="H64" s="75"/>
@@ -4640,14 +4623,14 @@
     </row>
     <row r="65" spans="1:13" ht="21" customHeight="1">
       <c r="A65" s="72" t="s">
-        <v>304</v>
-      </c>
-      <c r="B65" s="93"/>
-      <c r="C65" s="93"/>
-      <c r="D65" s="93"/>
-      <c r="E65" s="93"/>
+        <v>302</v>
+      </c>
+      <c r="B65" s="95"/>
+      <c r="C65" s="95"/>
+      <c r="D65" s="95"/>
+      <c r="E65" s="95"/>
       <c r="F65" s="73" t="s">
-        <v>149</v>
+        <v>289</v>
       </c>
       <c r="G65" s="75"/>
       <c r="H65" s="75"/>
@@ -4655,20 +4638,24 @@
       <c r="J65" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="K65" s="69"/>
+      <c r="K65" s="69" t="s">
+        <v>290</v>
+      </c>
       <c r="L65" s="68"/>
       <c r="M65" s="69"/>
     </row>
     <row r="66" spans="1:13" ht="21" customHeight="1">
       <c r="A66" s="72" t="s">
-        <v>306</v>
-      </c>
-      <c r="B66" s="93"/>
-      <c r="C66" s="93"/>
-      <c r="D66" s="93"/>
-      <c r="E66" s="93"/>
+        <v>304</v>
+      </c>
+      <c r="B66" s="95"/>
+      <c r="C66" s="95"/>
+      <c r="D66" s="95"/>
+      <c r="E66" s="73" t="s">
+        <v>292</v>
+      </c>
       <c r="F66" s="73" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="G66" s="75"/>
       <c r="H66" s="75"/>
@@ -4677,23 +4664,23 @@
         <v>8</v>
       </c>
       <c r="K66" s="69" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="L66" s="68"/>
       <c r="M66" s="69"/>
     </row>
     <row r="67" spans="1:13" ht="21" customHeight="1">
       <c r="A67" s="72" t="s">
-        <v>308</v>
-      </c>
-      <c r="B67" s="93"/>
-      <c r="C67" s="93"/>
-      <c r="D67" s="93"/>
-      <c r="E67" s="73" t="s">
-        <v>294</v>
+        <v>306</v>
+      </c>
+      <c r="B67" s="95"/>
+      <c r="C67" s="95"/>
+      <c r="D67" s="95"/>
+      <c r="E67" s="99" t="s">
+        <v>296</v>
       </c>
       <c r="F67" s="73" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G67" s="75"/>
       <c r="H67" s="75"/>
@@ -4702,23 +4689,21 @@
         <v>8</v>
       </c>
       <c r="K67" s="69" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="L67" s="68"/>
       <c r="M67" s="69"/>
     </row>
     <row r="68" spans="1:13" ht="21" customHeight="1">
       <c r="A68" s="72" t="s">
-        <v>311</v>
-      </c>
-      <c r="B68" s="93"/>
-      <c r="C68" s="93"/>
-      <c r="D68" s="93"/>
-      <c r="E68" s="96" t="s">
-        <v>298</v>
-      </c>
+        <v>309</v>
+      </c>
+      <c r="B68" s="95"/>
+      <c r="C68" s="95"/>
+      <c r="D68" s="95"/>
+      <c r="E68" s="102"/>
       <c r="F68" s="73" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G68" s="75"/>
       <c r="H68" s="75"/>
@@ -4727,21 +4712,21 @@
         <v>8</v>
       </c>
       <c r="K68" s="69" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L68" s="68"/>
       <c r="M68" s="69"/>
     </row>
     <row r="69" spans="1:13" ht="21" customHeight="1">
       <c r="A69" s="72" t="s">
-        <v>315</v>
-      </c>
-      <c r="B69" s="93"/>
-      <c r="C69" s="93"/>
-      <c r="D69" s="93"/>
-      <c r="E69" s="97"/>
+        <v>313</v>
+      </c>
+      <c r="B69" s="95"/>
+      <c r="C69" s="95"/>
+      <c r="D69" s="95"/>
+      <c r="E69" s="102"/>
       <c r="F69" s="73" t="s">
-        <v>302</v>
+        <v>217</v>
       </c>
       <c r="G69" s="75"/>
       <c r="H69" s="75"/>
@@ -4757,14 +4742,14 @@
     </row>
     <row r="70" spans="1:13" ht="21" customHeight="1">
       <c r="A70" s="72" t="s">
-        <v>317</v>
-      </c>
-      <c r="B70" s="93"/>
-      <c r="C70" s="93"/>
-      <c r="D70" s="93"/>
-      <c r="E70" s="97"/>
+        <v>315</v>
+      </c>
+      <c r="B70" s="95"/>
+      <c r="C70" s="95"/>
+      <c r="D70" s="95"/>
+      <c r="E70" s="102"/>
       <c r="F70" s="73" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="G70" s="75"/>
       <c r="H70" s="75"/>
@@ -4780,14 +4765,14 @@
     </row>
     <row r="71" spans="1:13" ht="21" customHeight="1">
       <c r="A71" s="72" t="s">
-        <v>318</v>
-      </c>
-      <c r="B71" s="93"/>
-      <c r="C71" s="93"/>
-      <c r="D71" s="93"/>
-      <c r="E71" s="97"/>
+        <v>316</v>
+      </c>
+      <c r="B71" s="95"/>
+      <c r="C71" s="95"/>
+      <c r="D71" s="95"/>
+      <c r="E71" s="102"/>
       <c r="F71" s="73" t="s">
-        <v>221</v>
+        <v>307</v>
       </c>
       <c r="G71" s="75"/>
       <c r="H71" s="75"/>
@@ -4796,21 +4781,21 @@
         <v>8</v>
       </c>
       <c r="K71" s="69" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L71" s="68"/>
       <c r="M71" s="69"/>
     </row>
     <row r="72" spans="1:13" ht="21" customHeight="1">
       <c r="A72" s="72" t="s">
-        <v>321</v>
-      </c>
-      <c r="B72" s="93"/>
-      <c r="C72" s="93"/>
-      <c r="D72" s="93"/>
-      <c r="E72" s="97"/>
+        <v>319</v>
+      </c>
+      <c r="B72" s="95"/>
+      <c r="C72" s="95"/>
+      <c r="D72" s="95"/>
+      <c r="E72" s="102"/>
       <c r="F72" s="73" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G72" s="75"/>
       <c r="H72" s="75"/>
@@ -4819,21 +4804,23 @@
         <v>8</v>
       </c>
       <c r="K72" s="69" t="s">
-        <v>310</v>
-      </c>
-      <c r="L72" s="68"/>
+        <v>311</v>
+      </c>
+      <c r="L72" s="68" t="s">
+        <v>312</v>
+      </c>
       <c r="M72" s="69"/>
     </row>
     <row r="73" spans="1:13" ht="21" customHeight="1">
       <c r="A73" s="72" t="s">
-        <v>324</v>
-      </c>
-      <c r="B73" s="93"/>
-      <c r="C73" s="93"/>
-      <c r="D73" s="93"/>
-      <c r="E73" s="97"/>
-      <c r="F73" s="73" t="s">
-        <v>312</v>
+        <v>322</v>
+      </c>
+      <c r="B73" s="95"/>
+      <c r="C73" s="95"/>
+      <c r="D73" s="95"/>
+      <c r="E73" s="100"/>
+      <c r="F73" s="71" t="s">
+        <v>230</v>
       </c>
       <c r="G73" s="75"/>
       <c r="H73" s="75"/>
@@ -4842,74 +4829,72 @@
         <v>8</v>
       </c>
       <c r="K73" s="69" t="s">
-        <v>313</v>
-      </c>
-      <c r="L73" s="68" t="s">
         <v>314</v>
       </c>
+      <c r="L73" s="68"/>
       <c r="M73" s="69"/>
     </row>
     <row r="74" spans="1:13" ht="21" customHeight="1">
       <c r="A74" s="72" t="s">
-        <v>327</v>
-      </c>
-      <c r="B74" s="93"/>
-      <c r="C74" s="93"/>
-      <c r="D74" s="93"/>
-      <c r="E74" s="98"/>
-      <c r="F74" s="71" t="s">
-        <v>230</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="B74" s="94" t="s">
+        <v>21</v>
+      </c>
+      <c r="C74" s="94" t="s">
+        <v>139</v>
+      </c>
+      <c r="D74" s="94" t="s">
+        <v>21</v>
+      </c>
+      <c r="E74" s="75"/>
+      <c r="F74" s="75"/>
       <c r="G74" s="75"/>
       <c r="H74" s="75"/>
-      <c r="I74" s="68"/>
-      <c r="J74" s="76" t="s">
-        <v>8</v>
+      <c r="I74" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="J74" s="77" t="s">
+        <v>23</v>
       </c>
       <c r="K74" s="69" t="s">
-        <v>316</v>
+        <v>99</v>
       </c>
       <c r="L74" s="68"/>
       <c r="M74" s="69"/>
     </row>
     <row r="75" spans="1:13" ht="21" customHeight="1">
       <c r="A75" s="72" t="s">
-        <v>329</v>
-      </c>
-      <c r="B75" s="92" t="s">
-        <v>21</v>
-      </c>
-      <c r="C75" s="92" t="s">
-        <v>139</v>
-      </c>
-      <c r="D75" s="92" t="s">
-        <v>21</v>
-      </c>
-      <c r="E75" s="75"/>
+        <v>327</v>
+      </c>
+      <c r="B75" s="95"/>
+      <c r="C75" s="95"/>
+      <c r="D75" s="95"/>
+      <c r="E75" s="73" t="s">
+        <v>317</v>
+      </c>
       <c r="F75" s="75"/>
       <c r="G75" s="75"/>
       <c r="H75" s="75"/>
-      <c r="I75" s="68" t="s">
-        <v>22</v>
-      </c>
+      <c r="I75" s="68"/>
       <c r="J75" s="77" t="s">
         <v>23</v>
       </c>
       <c r="K75" s="69" t="s">
-        <v>99</v>
+        <v>318</v>
       </c>
       <c r="L75" s="68"/>
       <c r="M75" s="69"/>
     </row>
     <row r="76" spans="1:13" ht="21" customHeight="1">
       <c r="A76" s="72" t="s">
-        <v>332</v>
-      </c>
-      <c r="B76" s="93"/>
-      <c r="C76" s="93"/>
-      <c r="D76" s="93"/>
+        <v>330</v>
+      </c>
+      <c r="B76" s="95"/>
+      <c r="C76" s="95"/>
+      <c r="D76" s="95"/>
       <c r="E76" s="73" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F76" s="75"/>
       <c r="G76" s="75"/>
@@ -4919,20 +4904,20 @@
         <v>23</v>
       </c>
       <c r="K76" s="69" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="L76" s="68"/>
       <c r="M76" s="69"/>
     </row>
     <row r="77" spans="1:13" ht="21" customHeight="1">
       <c r="A77" s="72" t="s">
-        <v>334</v>
-      </c>
-      <c r="B77" s="93"/>
-      <c r="C77" s="93"/>
-      <c r="D77" s="93"/>
+        <v>332</v>
+      </c>
+      <c r="B77" s="95"/>
+      <c r="C77" s="95"/>
+      <c r="D77" s="95"/>
       <c r="E77" s="73" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F77" s="75"/>
       <c r="G77" s="75"/>
@@ -4942,20 +4927,20 @@
         <v>23</v>
       </c>
       <c r="K77" s="69" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="L77" s="68"/>
       <c r="M77" s="69"/>
     </row>
     <row r="78" spans="1:13" ht="21" customHeight="1">
       <c r="A78" s="72" t="s">
-        <v>335</v>
-      </c>
-      <c r="B78" s="93"/>
-      <c r="C78" s="93"/>
-      <c r="D78" s="93"/>
+        <v>333</v>
+      </c>
+      <c r="B78" s="95"/>
+      <c r="C78" s="95"/>
+      <c r="D78" s="95"/>
       <c r="E78" s="73" t="s">
-        <v>325</v>
+        <v>106</v>
       </c>
       <c r="F78" s="75"/>
       <c r="G78" s="75"/>
@@ -4972,15 +4957,17 @@
     </row>
     <row r="79" spans="1:13" ht="21" customHeight="1">
       <c r="A79" s="72" t="s">
-        <v>336</v>
-      </c>
-      <c r="B79" s="93"/>
-      <c r="C79" s="93"/>
-      <c r="D79" s="93"/>
+        <v>334</v>
+      </c>
+      <c r="B79" s="95"/>
+      <c r="C79" s="95"/>
+      <c r="D79" s="95"/>
       <c r="E79" s="73" t="s">
-        <v>106</v>
-      </c>
-      <c r="F79" s="75"/>
+        <v>308</v>
+      </c>
+      <c r="F79" s="71" t="s">
+        <v>328</v>
+      </c>
       <c r="G79" s="75"/>
       <c r="H79" s="75"/>
       <c r="I79" s="68"/>
@@ -4988,24 +4975,22 @@
         <v>23</v>
       </c>
       <c r="K79" s="69" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="L79" s="68"/>
       <c r="M79" s="69"/>
     </row>
     <row r="80" spans="1:13" ht="21" customHeight="1">
       <c r="A80" s="72" t="s">
-        <v>337</v>
-      </c>
-      <c r="B80" s="93"/>
-      <c r="C80" s="93"/>
-      <c r="D80" s="93"/>
+        <v>335</v>
+      </c>
+      <c r="B80" s="95"/>
+      <c r="C80" s="95"/>
+      <c r="D80" s="95"/>
       <c r="E80" s="73" t="s">
-        <v>310</v>
-      </c>
-      <c r="F80" s="71" t="s">
-        <v>330</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="F80" s="75"/>
       <c r="G80" s="75"/>
       <c r="H80" s="75"/>
       <c r="I80" s="68"/>
@@ -5020,42 +5005,42 @@
     </row>
     <row r="81" spans="1:13" ht="21" customHeight="1">
       <c r="A81" s="72" t="s">
-        <v>338</v>
-      </c>
-      <c r="B81" s="93"/>
-      <c r="C81" s="93"/>
-      <c r="D81" s="93"/>
+        <v>336</v>
+      </c>
+      <c r="B81" s="99" t="s">
+        <v>25</v>
+      </c>
+      <c r="C81" s="99" t="s">
+        <v>139</v>
+      </c>
+      <c r="D81" s="99" t="s">
+        <v>25</v>
+      </c>
       <c r="E81" s="73" t="s">
-        <v>194</v>
+        <v>380</v>
       </c>
       <c r="F81" s="75"/>
       <c r="G81" s="75"/>
       <c r="H81" s="75"/>
       <c r="I81" s="68"/>
-      <c r="J81" s="77" t="s">
-        <v>23</v>
+      <c r="J81" s="76" t="s">
+        <v>8</v>
       </c>
       <c r="K81" s="69" t="s">
-        <v>333</v>
+        <v>381</v>
       </c>
       <c r="L81" s="68"/>
       <c r="M81" s="69"/>
     </row>
-    <row r="82" spans="1:13" ht="21" customHeight="1">
+    <row r="82" spans="1:13" s="67" customFormat="1" ht="21" customHeight="1">
       <c r="A82" s="72" t="s">
-        <v>339</v>
-      </c>
-      <c r="B82" s="96" t="s">
-        <v>25</v>
-      </c>
-      <c r="C82" s="96" t="s">
-        <v>139</v>
-      </c>
-      <c r="D82" s="96" t="s">
-        <v>25</v>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="B82" s="100"/>
+      <c r="C82" s="100"/>
+      <c r="D82" s="100"/>
       <c r="E82" s="73" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F82" s="75"/>
       <c r="G82" s="75"/>
@@ -5064,63 +5049,43 @@
       <c r="J82" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="K82" s="69" t="s">
-        <v>386</v>
-      </c>
+      <c r="K82" s="69"/>
       <c r="L82" s="68"/>
       <c r="M82" s="69"/>
     </row>
-    <row r="83" spans="1:13" s="104" customFormat="1" ht="21" customHeight="1">
+    <row r="83" spans="1:13" ht="21" customHeight="1">
       <c r="A83" s="72" t="s">
+        <v>339</v>
+      </c>
+      <c r="B83" s="71" t="s">
+        <v>378</v>
+      </c>
+      <c r="C83" s="71" t="s">
+        <v>379</v>
+      </c>
+      <c r="D83" s="78" t="s">
+        <v>340</v>
+      </c>
+      <c r="E83" s="73" t="s">
         <v>341</v>
       </c>
-      <c r="B83" s="98"/>
-      <c r="C83" s="98"/>
-      <c r="D83" s="98"/>
-      <c r="E83" s="73" t="s">
-        <v>389</v>
-      </c>
-      <c r="F83" s="75"/>
-      <c r="G83" s="75"/>
-      <c r="H83" s="75"/>
-      <c r="I83" s="68"/>
+      <c r="F83" s="73" t="s">
+        <v>386</v>
+      </c>
+      <c r="G83" s="73"/>
+      <c r="H83" s="73"/>
+      <c r="I83" s="75"/>
       <c r="J83" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="K83" s="69"/>
-      <c r="L83" s="68"/>
+      <c r="K83" s="69" t="s">
+        <v>385</v>
+      </c>
+      <c r="L83" s="75"/>
       <c r="M83" s="69"/>
     </row>
-    <row r="84" spans="1:13" ht="21" customHeight="1">
-      <c r="A84" s="72" t="s">
-        <v>370</v>
-      </c>
-      <c r="B84" s="71" t="s">
-        <v>383</v>
-      </c>
-      <c r="C84" s="71" t="s">
-        <v>384</v>
-      </c>
-      <c r="D84" s="105" t="s">
-        <v>342</v>
-      </c>
-      <c r="E84" s="73" t="s">
-        <v>343</v>
-      </c>
-      <c r="F84" s="107" t="s">
-        <v>391</v>
-      </c>
-      <c r="G84" s="73"/>
-      <c r="H84" s="73"/>
-      <c r="I84" s="75"/>
-      <c r="J84" s="76" t="s">
-        <v>8</v>
-      </c>
-      <c r="K84" s="69" t="s">
-        <v>390</v>
-      </c>
-      <c r="L84" s="75"/>
-      <c r="M84" s="69"/>
+    <row r="84" spans="1:13" ht="15.75" customHeight="1">
+      <c r="J84" s="11"/>
     </row>
     <row r="85" spans="1:13" ht="15.75" customHeight="1">
       <c r="J85" s="11"/>
@@ -5539,9 +5504,7 @@
     <row r="223" spans="10:10" ht="15.75" customHeight="1">
       <c r="J223" s="11"/>
     </row>
-    <row r="224" spans="10:10" ht="15.75" customHeight="1">
-      <c r="J224" s="11"/>
-    </row>
+    <row r="224" spans="10:10" ht="15.75" customHeight="1"/>
     <row r="225" ht="15.75" customHeight="1"/>
     <row r="226" ht="15.75" customHeight="1"/>
     <row r="227" ht="15.75" customHeight="1"/>
@@ -6302,49 +6265,48 @@
     <row r="982" ht="15.75" customHeight="1"/>
     <row r="983" ht="15.75" customHeight="1"/>
     <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A5:L82" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A5:L81" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="39">
-    <mergeCell ref="E9:E14"/>
-    <mergeCell ref="B82:B83"/>
-    <mergeCell ref="C82:C83"/>
-    <mergeCell ref="D82:D83"/>
+    <mergeCell ref="C8:C20"/>
+    <mergeCell ref="C60:C73"/>
+    <mergeCell ref="D74:D80"/>
+    <mergeCell ref="D8:D20"/>
+    <mergeCell ref="D60:D73"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="D81:D82"/>
     <mergeCell ref="F30:F31"/>
-    <mergeCell ref="B61:B74"/>
+    <mergeCell ref="B60:B73"/>
+    <mergeCell ref="D41:D59"/>
+    <mergeCell ref="C21:C40"/>
+    <mergeCell ref="E54:E59"/>
+    <mergeCell ref="E67:E73"/>
+    <mergeCell ref="B74:B80"/>
+    <mergeCell ref="E50:E52"/>
+    <mergeCell ref="E35:E40"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="F28:F29"/>
     <mergeCell ref="E44:E48"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="E30:E34"/>
-    <mergeCell ref="D41:D60"/>
-    <mergeCell ref="C21:C40"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="E9:E14"/>
     <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C75:C81"/>
+    <mergeCell ref="C74:C80"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="D21:D40"/>
     <mergeCell ref="F25:F26"/>
     <mergeCell ref="F44:F45"/>
-    <mergeCell ref="C41:C60"/>
+    <mergeCell ref="C41:C59"/>
     <mergeCell ref="E22:E29"/>
     <mergeCell ref="B8:B20"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="E63:E66"/>
-    <mergeCell ref="B41:B60"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="B41:B59"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B21:B40"/>
     <mergeCell ref="E15:E20"/>
-    <mergeCell ref="E35:E40"/>
-    <mergeCell ref="E55:E60"/>
-    <mergeCell ref="E68:E74"/>
-    <mergeCell ref="B75:B81"/>
-    <mergeCell ref="C8:C20"/>
-    <mergeCell ref="C61:C74"/>
-    <mergeCell ref="D75:D81"/>
-    <mergeCell ref="D8:D20"/>
-    <mergeCell ref="D61:D74"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="E50:E53"/>
   </mergeCells>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -6370,7 +6332,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="35" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
@@ -6385,30 +6347,30 @@
       <c r="L1" s="20"/>
     </row>
     <row r="2" spans="1:12" ht="22" customHeight="1">
-      <c r="A2" s="103" t="s">
-        <v>345</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
+      <c r="A2" s="105" t="s">
+        <v>343</v>
+      </c>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
     </row>
     <row r="3" spans="1:12" ht="23" customHeight="1"/>
     <row r="4" spans="1:12" ht="24" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>348</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="42" customHeight="1">
@@ -6416,33 +6378,33 @@
         <v>142</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="42" customHeight="1">
       <c r="A6" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>354</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>355</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>356</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>18</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="42" customHeight="1">
@@ -6450,55 +6412,55 @@
         <v>102</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="42" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>361</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>362</v>
-      </c>
       <c r="E8" s="3" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="42" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="E9" s="2" t="s">
         <v>364</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>365</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1">
       <c r="E11" s="35" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>